<commit_message>
Revisão de alguns componentes e serviços para arrumar um problema na atualização da tabela de previsoes, alteração do gerado de relatorio para incluir o mapa do IMET e tambem os gráficos, inclusao de uma função para gerar a imagem do infoclima, esta imagem vai para o relatorio em excel.
</commit_message>
<xml_diff>
--- a/templates/excel/ReportTemplate.xlsx
+++ b/templates/excel/ReportTemplate.xlsx
@@ -2,22 +2,22 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <workbookPr codeName="EstaPastaDeTrabalho" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Emerson\Documents\MBA\Projetos\weather-forecast\templates\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FD17177-F1DE-470C-997D-466B3E690F80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83CE026B-15F6-4969-BD3A-2DD93AC81677}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="23280" windowHeight="12480" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tempo Agora" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="Abreviatura" hidden="1">#REF!</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Tempo Agora'!$A$1:$E$28</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Tempo Agora'!$A$1:$G$46</definedName>
     <definedName name="_xlnm.Recorder">#REF!</definedName>
     <definedName name="HSEAccidentsTable">OFFSET(#REF!,0,0,COUNTA(#REF!),5)</definedName>
     <definedName name="index_areaER">#REF!</definedName>
@@ -26,9 +26,23 @@
     <definedName name="NomePrograma">#REF!</definedName>
     <definedName name="RdoData">#REF!</definedName>
     <definedName name="sss">OFFSET(#REF!,0,0,COUNTA(#REF!),5)</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">'Tempo Agora'!$1:$1</definedName>
     <definedName name="XXX">#REF!</definedName>
   </definedNames>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -54,7 +68,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -83,25 +97,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="12"/>
-      <color rgb="FF202124"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="14"/>
-      <color rgb="FF202124"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="30"/>
-      <color rgb="FFF0622E"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
       <u/>
       <sz val="12"/>
       <color theme="1"/>
@@ -112,27 +107,20 @@
     <font>
       <b/>
       <sz val="14"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
+      <color rgb="FF202124"/>
+      <name val="Arial"/>
       <family val="2"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF8FBFF"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="14">
+  <borders count="19">
     <border>
       <left/>
       <right/>
@@ -194,7 +182,7 @@
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
+      <left style="thin">
         <color indexed="64"/>
       </left>
       <right style="thin">
@@ -203,7 +191,33 @@
       <top style="thin">
         <color indexed="64"/>
       </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
       <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
@@ -224,10 +238,10 @@
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
+      <left style="thin">
         <color indexed="64"/>
       </left>
-      <right style="thin">
+      <right style="medium">
         <color indexed="64"/>
       </right>
       <top style="thin">
@@ -239,29 +253,62 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
+      <left/>
       <right style="thin">
         <color indexed="64"/>
       </right>
       <top style="thin">
         <color indexed="64"/>
       </top>
-      <bottom style="medium">
+      <bottom style="thin">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
+      <left/>
+      <right style="thin">
         <color indexed="64"/>
       </right>
       <top style="thin">
         <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
       </top>
       <bottom style="medium">
         <color indexed="64"/>
@@ -274,7 +321,7 @@
       </left>
       <right/>
       <top/>
-      <bottom style="thin">
+      <bottom style="medium">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
@@ -283,22 +330,20 @@
       <left/>
       <right/>
       <top/>
-      <bottom style="thin">
+      <bottom style="medium">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
+      <left/>
       <right style="medium">
         <color indexed="64"/>
       </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -308,61 +353,48 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -387,44 +419,61 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>1465384</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>210572</xdr:rowOff>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>1188982</xdr:colOff>
+      <xdr:row>34</xdr:row>
+      <xdr:rowOff>5</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>4417104</xdr:colOff>
-      <xdr:row>10</xdr:row>
-      <xdr:rowOff>106661</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>1913203</xdr:colOff>
+      <xdr:row>45</xdr:row>
+      <xdr:rowOff>75047</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="64" name="Imagem 63">
+        <xdr:cNvPr id="72" name="Imagem 71" descr="0">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{706597D0-C0EB-2128-1227-7468E58E1FF8}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{FDADAA38-4A00-C257-0D4A-1B8EBB57BF8A}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
         <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </xdr:blipFill>
-      <xdr:spPr>
+      <xdr:spPr bwMode="auto">
         <a:xfrm>
-          <a:off x="5026269" y="210572"/>
-          <a:ext cx="2951720" cy="2914781"/>
+          <a:off x="4828189" y="16277902"/>
+          <a:ext cx="2274497" cy="2242800"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>
@@ -749,238 +798,461 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr>
-    <pageSetUpPr fitToPage="1"/>
-  </sheetPr>
-  <dimension ref="A1:E28"/>
+  <sheetPr codeName="Planilha1"/>
+  <dimension ref="A1:G46"/>
   <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.5" customWidth="1"/>
-    <col min="2" max="2" width="9.625" customWidth="1"/>
-    <col min="3" max="3" width="9.875" customWidth="1"/>
-    <col min="4" max="4" width="18.75" customWidth="1"/>
-    <col min="5" max="5" width="64.625" customWidth="1"/>
+    <col min="1" max="1" width="0.875" customWidth="1"/>
+    <col min="2" max="2" width="8.5" customWidth="1"/>
+    <col min="3" max="3" width="9.625" customWidth="1"/>
+    <col min="4" max="4" width="9.875" customWidth="1"/>
+    <col min="5" max="5" width="18.75" customWidth="1"/>
+    <col min="6" max="6" width="20.375" customWidth="1"/>
+    <col min="7" max="7" width="40.25" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="15"/>
+    <row r="1" spans="1:7" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="10"/>
       <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
       <c r="E1" s="17"/>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="3"/>
-      <c r="B2" s="21"/>
-      <c r="C2" s="21"/>
-      <c r="D2" s="21"/>
-      <c r="E2" s="4"/>
-    </row>
-    <row r="3" spans="1:5" ht="72" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="3"/>
-      <c r="B3" s="21"/>
-      <c r="C3" s="21"/>
-      <c r="D3" s="22"/>
-      <c r="E3" s="4"/>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="3"/>
-      <c r="B4" s="21"/>
-      <c r="C4" s="21"/>
-      <c r="D4" s="21"/>
-      <c r="E4" s="4"/>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="14"/>
-      <c r="B5" s="23"/>
-      <c r="C5" s="23"/>
-      <c r="D5" s="23"/>
-      <c r="E5" s="5"/>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="3"/>
-      <c r="B6" s="24"/>
-      <c r="C6" s="21"/>
-      <c r="D6" s="21"/>
-      <c r="E6" s="4"/>
-    </row>
-    <row r="7" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="25"/>
-      <c r="B7" s="26"/>
-      <c r="C7" s="26"/>
-      <c r="D7" s="27"/>
-      <c r="E7" s="5"/>
-    </row>
-    <row r="8" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="25"/>
-      <c r="B8" s="26"/>
-      <c r="C8" s="26"/>
-      <c r="D8" s="27"/>
-      <c r="E8" s="5"/>
-    </row>
-    <row r="9" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="25"/>
-      <c r="B9" s="26"/>
-      <c r="C9" s="26"/>
-      <c r="D9" s="27"/>
-      <c r="E9" s="5"/>
-    </row>
-    <row r="10" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="25"/>
-      <c r="B10" s="26"/>
-      <c r="C10" s="26"/>
-      <c r="D10" s="27"/>
-      <c r="E10" s="5"/>
-    </row>
-    <row r="11" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="25"/>
-      <c r="B11" s="26"/>
-      <c r="C11" s="26"/>
-      <c r="D11" s="27"/>
-      <c r="E11" s="5"/>
-    </row>
-    <row r="12" spans="1:5" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="20"/>
-      <c r="B12" s="11"/>
-      <c r="C12" s="11"/>
-      <c r="D12" s="11"/>
-      <c r="E12" s="4"/>
-    </row>
-    <row r="13" spans="1:5" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="6" t="s">
+      <c r="F1" s="17"/>
+      <c r="G1" s="18"/>
+    </row>
+    <row r="2" spans="1:7" ht="242.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="1"/>
+      <c r="G2" s="2"/>
+    </row>
+    <row r="3" spans="1:7" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="11"/>
+      <c r="B3" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B13" s="1" t="s">
+      <c r="C3" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C13" s="1" t="s">
+      <c r="D3" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D13" s="1" t="s">
+      <c r="E3" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E13" s="7" t="s">
+      <c r="F3" s="19" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="14" spans="1:5" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="12"/>
-      <c r="B14" s="2"/>
-      <c r="C14" s="2"/>
-      <c r="D14" s="2"/>
-      <c r="E14" s="13"/>
-    </row>
-    <row r="15" spans="1:5" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="12"/>
-      <c r="B15" s="2"/>
-      <c r="C15" s="2"/>
-      <c r="D15" s="2"/>
-      <c r="E15" s="18"/>
-    </row>
-    <row r="16" spans="1:5" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="8"/>
-      <c r="B16" s="2"/>
-      <c r="C16" s="2"/>
-      <c r="D16" s="2"/>
-      <c r="E16" s="18"/>
-    </row>
-    <row r="17" spans="1:5" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="8"/>
-      <c r="B17" s="2"/>
-      <c r="C17" s="2"/>
-      <c r="D17" s="2"/>
-      <c r="E17" s="18"/>
-    </row>
-    <row r="18" spans="1:5" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="8"/>
-      <c r="B18" s="2"/>
-      <c r="C18" s="2"/>
-      <c r="D18" s="2"/>
-      <c r="E18" s="18"/>
-    </row>
-    <row r="19" spans="1:5" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="8"/>
-      <c r="B19" s="2"/>
-      <c r="C19" s="2"/>
-      <c r="D19" s="2"/>
-      <c r="E19" s="18"/>
-    </row>
-    <row r="20" spans="1:5" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="8"/>
-      <c r="B20" s="2"/>
-      <c r="C20" s="2"/>
-      <c r="D20" s="2"/>
-      <c r="E20" s="18"/>
-    </row>
-    <row r="21" spans="1:5" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="8"/>
-      <c r="B21" s="2"/>
-      <c r="C21" s="2"/>
-      <c r="D21" s="2"/>
-      <c r="E21" s="18"/>
-    </row>
-    <row r="22" spans="1:5" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="8"/>
-      <c r="B22" s="2"/>
-      <c r="C22" s="2"/>
-      <c r="D22" s="2"/>
-      <c r="E22" s="18"/>
-    </row>
-    <row r="23" spans="1:5" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="8"/>
-      <c r="B23" s="2"/>
-      <c r="C23" s="2"/>
-      <c r="D23" s="2"/>
-      <c r="E23" s="18"/>
-    </row>
-    <row r="24" spans="1:5" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="8"/>
-      <c r="B24" s="2"/>
-      <c r="C24" s="2"/>
-      <c r="D24" s="2"/>
-      <c r="E24" s="18"/>
-    </row>
-    <row r="25" spans="1:5" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="8"/>
-      <c r="B25" s="2"/>
-      <c r="C25" s="2"/>
-      <c r="D25" s="2"/>
-      <c r="E25" s="18"/>
-    </row>
-    <row r="26" spans="1:5" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="8"/>
-      <c r="B26" s="2"/>
-      <c r="C26" s="2"/>
-      <c r="D26" s="2"/>
-      <c r="E26" s="18"/>
-    </row>
-    <row r="27" spans="1:5" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="8"/>
-      <c r="B27" s="2"/>
-      <c r="C27" s="2"/>
-      <c r="D27" s="2"/>
-      <c r="E27" s="18"/>
-    </row>
-    <row r="28" spans="1:5" ht="48" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="9"/>
-      <c r="B28" s="10"/>
-      <c r="C28" s="10"/>
-      <c r="D28" s="10"/>
-      <c r="E28" s="19"/>
+      <c r="G3" s="15"/>
+    </row>
+    <row r="4" spans="1:7" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="11"/>
+      <c r="B4" s="7"/>
+      <c r="C4" s="4"/>
+      <c r="D4" s="4"/>
+      <c r="E4" s="4"/>
+      <c r="F4" s="25"/>
+      <c r="G4" s="26"/>
+    </row>
+    <row r="5" spans="1:7" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="11"/>
+      <c r="B5" s="7"/>
+      <c r="C5" s="4"/>
+      <c r="D5" s="4"/>
+      <c r="E5" s="4"/>
+      <c r="F5" s="25"/>
+      <c r="G5" s="26"/>
+    </row>
+    <row r="6" spans="1:7" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="11"/>
+      <c r="B6" s="8"/>
+      <c r="C6" s="4"/>
+      <c r="D6" s="4"/>
+      <c r="E6" s="4"/>
+      <c r="F6" s="25"/>
+      <c r="G6" s="26"/>
+    </row>
+    <row r="7" spans="1:7" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="11"/>
+      <c r="B7" s="8"/>
+      <c r="C7" s="4"/>
+      <c r="D7" s="4"/>
+      <c r="E7" s="4"/>
+      <c r="F7" s="25"/>
+      <c r="G7" s="26"/>
+    </row>
+    <row r="8" spans="1:7" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="11"/>
+      <c r="B8" s="8"/>
+      <c r="C8" s="4"/>
+      <c r="D8" s="4"/>
+      <c r="E8" s="4"/>
+      <c r="F8" s="25"/>
+      <c r="G8" s="26"/>
+    </row>
+    <row r="9" spans="1:7" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="11"/>
+      <c r="B9" s="8"/>
+      <c r="C9" s="4"/>
+      <c r="D9" s="4"/>
+      <c r="E9" s="4"/>
+      <c r="F9" s="25"/>
+      <c r="G9" s="26"/>
+    </row>
+    <row r="10" spans="1:7" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="11"/>
+      <c r="B10" s="8"/>
+      <c r="C10" s="4"/>
+      <c r="D10" s="4"/>
+      <c r="E10" s="4"/>
+      <c r="F10" s="25"/>
+      <c r="G10" s="26"/>
+    </row>
+    <row r="11" spans="1:7" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="11"/>
+      <c r="B11" s="8"/>
+      <c r="C11" s="4"/>
+      <c r="D11" s="4"/>
+      <c r="E11" s="4"/>
+      <c r="F11" s="25"/>
+      <c r="G11" s="26"/>
+    </row>
+    <row r="12" spans="1:7" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="11"/>
+      <c r="B12" s="8"/>
+      <c r="C12" s="4"/>
+      <c r="D12" s="4"/>
+      <c r="E12" s="4"/>
+      <c r="F12" s="25"/>
+      <c r="G12" s="26"/>
+    </row>
+    <row r="13" spans="1:7" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="11"/>
+      <c r="B13" s="8"/>
+      <c r="C13" s="4"/>
+      <c r="D13" s="4"/>
+      <c r="E13" s="4"/>
+      <c r="F13" s="25"/>
+      <c r="G13" s="26"/>
+    </row>
+    <row r="14" spans="1:7" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="11"/>
+      <c r="B14" s="8"/>
+      <c r="C14" s="4"/>
+      <c r="D14" s="4"/>
+      <c r="E14" s="4"/>
+      <c r="F14" s="25"/>
+      <c r="G14" s="26"/>
+    </row>
+    <row r="15" spans="1:7" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="11"/>
+      <c r="B15" s="8"/>
+      <c r="C15" s="4"/>
+      <c r="D15" s="4"/>
+      <c r="E15" s="4"/>
+      <c r="F15" s="25"/>
+      <c r="G15" s="26"/>
+    </row>
+    <row r="16" spans="1:7" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="11"/>
+      <c r="B16" s="8"/>
+      <c r="C16" s="4"/>
+      <c r="D16" s="4"/>
+      <c r="E16" s="4"/>
+      <c r="F16" s="25"/>
+      <c r="G16" s="26"/>
+    </row>
+    <row r="17" spans="1:7" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="11"/>
+      <c r="B17" s="8"/>
+      <c r="C17" s="4"/>
+      <c r="D17" s="4"/>
+      <c r="E17" s="4"/>
+      <c r="F17" s="25"/>
+      <c r="G17" s="26"/>
+    </row>
+    <row r="18" spans="1:7" ht="48" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="12"/>
+      <c r="B18" s="9"/>
+      <c r="C18" s="5"/>
+      <c r="D18" s="5"/>
+      <c r="E18" s="5"/>
+      <c r="F18" s="27"/>
+      <c r="G18" s="28"/>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A19" s="10"/>
+      <c r="B19" s="13"/>
+      <c r="C19" s="13"/>
+      <c r="D19" s="13"/>
+      <c r="E19" s="13"/>
+      <c r="F19" s="13"/>
+      <c r="G19" s="14"/>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A20" s="1"/>
+      <c r="B20" s="20"/>
+      <c r="C20" s="20"/>
+      <c r="D20" s="20"/>
+      <c r="E20" s="20"/>
+      <c r="F20" s="20"/>
+      <c r="G20" s="2"/>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A21" s="1"/>
+      <c r="B21" s="20"/>
+      <c r="C21" s="20"/>
+      <c r="D21" s="20"/>
+      <c r="E21" s="20"/>
+      <c r="F21" s="20"/>
+      <c r="G21" s="2"/>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A22" s="1"/>
+      <c r="B22" s="20"/>
+      <c r="C22" s="20"/>
+      <c r="D22" s="20"/>
+      <c r="E22" s="20"/>
+      <c r="F22" s="20"/>
+      <c r="G22" s="2"/>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A23" s="1"/>
+      <c r="B23" s="20"/>
+      <c r="C23" s="20"/>
+      <c r="D23" s="20"/>
+      <c r="E23" s="20"/>
+      <c r="F23" s="20"/>
+      <c r="G23" s="2"/>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A24" s="1"/>
+      <c r="B24" s="20"/>
+      <c r="C24" s="20"/>
+      <c r="D24" s="20"/>
+      <c r="E24" s="20"/>
+      <c r="F24" s="20"/>
+      <c r="G24" s="2"/>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A25" s="1"/>
+      <c r="B25" s="20"/>
+      <c r="C25" s="20"/>
+      <c r="D25" s="20"/>
+      <c r="E25" s="20"/>
+      <c r="F25" s="20"/>
+      <c r="G25" s="2"/>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A26" s="1"/>
+      <c r="B26" s="20"/>
+      <c r="C26" s="20"/>
+      <c r="D26" s="20"/>
+      <c r="E26" s="20"/>
+      <c r="F26" s="20"/>
+      <c r="G26" s="2"/>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A27" s="1"/>
+      <c r="B27" s="20"/>
+      <c r="C27" s="20"/>
+      <c r="D27" s="20"/>
+      <c r="E27" s="20"/>
+      <c r="F27" s="20"/>
+      <c r="G27" s="2"/>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A28" s="1"/>
+      <c r="B28" s="20"/>
+      <c r="C28" s="20"/>
+      <c r="D28" s="20"/>
+      <c r="E28" s="20"/>
+      <c r="F28" s="20"/>
+      <c r="G28" s="2"/>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A29" s="1"/>
+      <c r="B29" s="20"/>
+      <c r="C29" s="20"/>
+      <c r="D29" s="20"/>
+      <c r="E29" s="20"/>
+      <c r="F29" s="20"/>
+      <c r="G29" s="2"/>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A30" s="1"/>
+      <c r="B30" s="20"/>
+      <c r="C30" s="20"/>
+      <c r="D30" s="20"/>
+      <c r="E30" s="20"/>
+      <c r="F30" s="20"/>
+      <c r="G30" s="2"/>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A31" s="1"/>
+      <c r="B31" s="20"/>
+      <c r="C31" s="20"/>
+      <c r="D31" s="20"/>
+      <c r="E31" s="20"/>
+      <c r="F31" s="20"/>
+      <c r="G31" s="21"/>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A32" s="1"/>
+      <c r="B32" s="20"/>
+      <c r="C32" s="20"/>
+      <c r="D32" s="20"/>
+      <c r="E32" s="20"/>
+      <c r="F32" s="20"/>
+      <c r="G32" s="2"/>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A33" s="1"/>
+      <c r="B33" s="20"/>
+      <c r="C33" s="20"/>
+      <c r="D33" s="20"/>
+      <c r="E33" s="20"/>
+      <c r="F33" s="20"/>
+      <c r="G33" s="2"/>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A34" s="1"/>
+      <c r="B34" s="20"/>
+      <c r="C34" s="20"/>
+      <c r="D34" s="20"/>
+      <c r="E34" s="20"/>
+      <c r="F34" s="20"/>
+      <c r="G34" s="2"/>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A35" s="1"/>
+      <c r="B35" s="20"/>
+      <c r="C35" s="20"/>
+      <c r="D35" s="20"/>
+      <c r="E35" s="20"/>
+      <c r="F35" s="20"/>
+      <c r="G35" s="2"/>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A36" s="1"/>
+      <c r="B36" s="20"/>
+      <c r="C36" s="20"/>
+      <c r="D36" s="20"/>
+      <c r="E36" s="20"/>
+      <c r="F36" s="20"/>
+      <c r="G36" s="2"/>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A37" s="1"/>
+      <c r="B37" s="20"/>
+      <c r="C37" s="20"/>
+      <c r="D37" s="20"/>
+      <c r="E37" s="20"/>
+      <c r="F37" s="20"/>
+      <c r="G37" s="2"/>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A38" s="1"/>
+      <c r="B38" s="20"/>
+      <c r="C38" s="20"/>
+      <c r="D38" s="20"/>
+      <c r="E38" s="20"/>
+      <c r="F38" s="20"/>
+      <c r="G38" s="2"/>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A39" s="1"/>
+      <c r="B39" s="20"/>
+      <c r="C39" s="20"/>
+      <c r="D39" s="20"/>
+      <c r="E39" s="20"/>
+      <c r="F39" s="20"/>
+      <c r="G39" s="2"/>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A40" s="1"/>
+      <c r="B40" s="20"/>
+      <c r="C40" s="20"/>
+      <c r="D40" s="20"/>
+      <c r="E40" s="20"/>
+      <c r="F40" s="20"/>
+      <c r="G40" s="2"/>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A41" s="1"/>
+      <c r="B41" s="20"/>
+      <c r="C41" s="20"/>
+      <c r="D41" s="20"/>
+      <c r="E41" s="20"/>
+      <c r="F41" s="20"/>
+      <c r="G41" s="2"/>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A42" s="1"/>
+      <c r="B42" s="20"/>
+      <c r="C42" s="20"/>
+      <c r="D42" s="20"/>
+      <c r="E42" s="20"/>
+      <c r="F42" s="20"/>
+      <c r="G42" s="2"/>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A43" s="1"/>
+      <c r="B43" s="20"/>
+      <c r="C43" s="20"/>
+      <c r="D43" s="20"/>
+      <c r="E43" s="20"/>
+      <c r="F43" s="20"/>
+      <c r="G43" s="2"/>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A44" s="1"/>
+      <c r="B44" s="20"/>
+      <c r="C44" s="20"/>
+      <c r="D44" s="20"/>
+      <c r="E44" s="20"/>
+      <c r="F44" s="20"/>
+      <c r="G44" s="2"/>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A45" s="1"/>
+      <c r="B45" s="20"/>
+      <c r="C45" s="20"/>
+      <c r="D45" s="20"/>
+      <c r="E45" s="20"/>
+      <c r="F45" s="20"/>
+      <c r="G45" s="2"/>
+    </row>
+    <row r="46" spans="1:7" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A46" s="22"/>
+      <c r="B46" s="23"/>
+      <c r="C46" s="23"/>
+      <c r="D46" s="23"/>
+      <c r="E46" s="23"/>
+      <c r="F46" s="23"/>
+      <c r="G46" s="24"/>
     </row>
   </sheetData>
-  <mergeCells count="7">
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A7:C7"/>
-    <mergeCell ref="A10:C10"/>
-    <mergeCell ref="A5:D5"/>
-    <mergeCell ref="A11:C11"/>
-    <mergeCell ref="A8:C8"/>
-    <mergeCell ref="A9:C9"/>
+  <mergeCells count="17">
+    <mergeCell ref="F10:G10"/>
+    <mergeCell ref="F16:G16"/>
+    <mergeCell ref="F5:G5"/>
+    <mergeCell ref="B1:G1"/>
+    <mergeCell ref="F18:G18"/>
+    <mergeCell ref="F6:G6"/>
+    <mergeCell ref="F14:G14"/>
+    <mergeCell ref="F13:G13"/>
+    <mergeCell ref="F17:G17"/>
+    <mergeCell ref="F9:G9"/>
+    <mergeCell ref="F7:G7"/>
+    <mergeCell ref="F8:G8"/>
+    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="F4:G4"/>
+    <mergeCell ref="F11:G11"/>
+    <mergeCell ref="F12:G12"/>
+    <mergeCell ref="F15:G15"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
-  <pageMargins left="0.39370078740157483" right="0.19685039370078741" top="0.39370078740157483" bottom="0.39370078740157483" header="0.11811023622047245" footer="0.11811023622047245"/>
-  <pageSetup paperSize="9" scale="73" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
+  <pageMargins left="0.19685039370078741" right="0.19685039370078741" top="0.39370078740157483" bottom="0.39370078740157483" header="0.11811023622047245" footer="0.11811023622047245"/>
+  <pageSetup paperSize="9" scale="73" fitToHeight="2" orientation="portrait" r:id="rId1"/>
   <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Alteracao do layout do relatório em excel, alteração do dos gráficos para para fixar o layout dos gráficos, alteração do layout dos graficos para irem com os valores nos rotulos, alteração de algumas funcoes para facilitar a colocação das informações no cabeçalho e no rodapé do relatorio em excel.
</commit_message>
<xml_diff>
--- a/templates/excel/ReportTemplate.xlsx
+++ b/templates/excel/ReportTemplate.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Emerson\Documents\MBA\Projetos\weather-forecast\templates\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2629F0C7-DC81-4F82-B4F5-970127E9028B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A0CC8EF-2EA0-4675-B44A-9BE63B2778AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,7 +17,7 @@
   </sheets>
   <definedNames>
     <definedName name="Abreviatura" hidden="1">#REF!</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Tempo Agora'!$A$1:$H$46</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Tempo Agora'!$A$1:$H$19,'Tempo Agora'!$J$1:$U$19</definedName>
     <definedName name="_xlnm.Recorder">#REF!</definedName>
     <definedName name="HSEAccidentsTable">OFFSET(#REF!,0,0,COUNTA(#REF!),5)</definedName>
     <definedName name="index_areaER">#REF!</definedName>
@@ -26,7 +26,7 @@
     <definedName name="NomePrograma">#REF!</definedName>
     <definedName name="RdoData">#REF!</definedName>
     <definedName name="sss">OFFSET(#REF!,0,0,COUNTA(#REF!),5)</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="0">'Tempo Agora'!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">'Tempo Agora'!$2:$2</definedName>
     <definedName name="XXX">#REF!</definedName>
   </definedNames>
   <calcPr calcId="0"/>
@@ -55,7 +55,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -98,6 +98,20 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <i/>
+      <sz val="8"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -107,7 +121,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="15">
+  <borders count="16">
     <border>
       <left/>
       <right/>
@@ -186,10 +200,12 @@
         <color indexed="64"/>
       </left>
       <right/>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -200,50 +216,6 @@
       <top style="thin">
         <color auto="1"/>
       </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top/>
       <bottom style="medium">
         <color indexed="64"/>
       </bottom>
@@ -271,6 +243,71 @@
       <bottom style="thin">
         <color indexed="64"/>
       </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
       <diagonal/>
     </border>
   </borders>
@@ -280,7 +317,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
@@ -295,23 +332,62 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -651,7 +727,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Planilha1"/>
-  <dimension ref="A1:H46"/>
+  <dimension ref="A1:U47"/>
   <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="0.875" customWidth="1"/>
@@ -662,332 +738,263 @@
     <col min="6" max="6" width="9.375" customWidth="1"/>
     <col min="7" max="7" width="18" customWidth="1"/>
     <col min="8" max="8" width="39.5" customWidth="1"/>
+    <col min="9" max="9" width="3.75" customWidth="1"/>
+    <col min="10" max="10" width="2.125" customWidth="1"/>
+    <col min="15" max="17" width="3" customWidth="1"/>
+    <col min="18" max="18" width="7.25" customWidth="1"/>
+    <col min="20" max="20" width="29.875" customWidth="1"/>
+    <col min="21" max="21" width="6.625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="8"/>
-      <c r="B1" s="18"/>
-      <c r="C1" s="19"/>
-      <c r="D1" s="19"/>
-      <c r="E1" s="19"/>
-      <c r="F1" s="19"/>
-      <c r="G1" s="19"/>
-      <c r="H1" s="20"/>
-    </row>
-    <row r="2" spans="1:8" ht="242.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:21" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="31"/>
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
+      <c r="E1" s="32"/>
+      <c r="F1" s="32"/>
+      <c r="G1" s="32"/>
+      <c r="H1" s="33"/>
+      <c r="J1" s="27"/>
+      <c r="K1" s="28"/>
+      <c r="L1" s="28"/>
+      <c r="M1" s="28"/>
+      <c r="N1" s="28"/>
+      <c r="O1" s="28"/>
+      <c r="P1" s="28"/>
+      <c r="Q1" s="28"/>
+      <c r="R1" s="28"/>
+      <c r="S1" s="28"/>
+      <c r="T1" s="28"/>
+      <c r="U1" s="28"/>
+    </row>
+    <row r="2" spans="1:21" ht="51" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1"/>
-      <c r="H2" s="2"/>
-    </row>
-    <row r="3" spans="1:8" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="9"/>
-      <c r="B3" s="5" t="s">
+      <c r="B2" s="20"/>
+      <c r="C2" s="15"/>
+      <c r="D2" s="16"/>
+      <c r="E2" s="19"/>
+      <c r="F2" s="13"/>
+      <c r="G2" s="12"/>
+      <c r="H2" s="14"/>
+      <c r="K2" s="20"/>
+      <c r="L2" s="17"/>
+      <c r="M2" s="18"/>
+      <c r="S2" s="12"/>
+      <c r="T2" s="34"/>
+      <c r="U2" s="34"/>
+    </row>
+    <row r="3" spans="1:21" ht="242.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="1"/>
+      <c r="H3" s="2"/>
+    </row>
+    <row r="4" spans="1:21" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="8"/>
+      <c r="B4" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C4" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="D4" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="E4" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="F3" s="21" t="s">
+      <c r="F4" s="29" t="s">
         <v>4</v>
       </c>
-      <c r="G3" s="16"/>
-      <c r="H3" s="17"/>
-    </row>
-    <row r="4" spans="1:8" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="9"/>
-      <c r="B4" s="6"/>
-      <c r="C4" s="4"/>
-      <c r="D4" s="4"/>
-      <c r="E4" s="4"/>
-      <c r="F4" s="15"/>
-      <c r="G4" s="16"/>
-      <c r="H4" s="17"/>
-    </row>
-    <row r="5" spans="1:8" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="9"/>
+      <c r="G4" s="22"/>
+      <c r="H4" s="23"/>
+    </row>
+    <row r="5" spans="1:21" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="8"/>
       <c r="B5" s="6"/>
       <c r="C5" s="4"/>
       <c r="D5" s="4"/>
       <c r="E5" s="4"/>
-      <c r="F5" s="15"/>
-      <c r="G5" s="16"/>
-      <c r="H5" s="17"/>
-    </row>
-    <row r="6" spans="1:8" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="9"/>
-      <c r="B6" s="7"/>
+      <c r="F5" s="21"/>
+      <c r="G5" s="22"/>
+      <c r="H5" s="23"/>
+    </row>
+    <row r="6" spans="1:21" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="8"/>
+      <c r="B6" s="6"/>
       <c r="C6" s="4"/>
       <c r="D6" s="4"/>
       <c r="E6" s="4"/>
-      <c r="F6" s="15"/>
-      <c r="G6" s="16"/>
-      <c r="H6" s="17"/>
-    </row>
-    <row r="7" spans="1:8" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="9"/>
+      <c r="F6" s="21"/>
+      <c r="G6" s="22"/>
+      <c r="H6" s="23"/>
+    </row>
+    <row r="7" spans="1:21" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="8"/>
       <c r="B7" s="7"/>
       <c r="C7" s="4"/>
       <c r="D7" s="4"/>
       <c r="E7" s="4"/>
-      <c r="F7" s="15"/>
-      <c r="G7" s="16"/>
-      <c r="H7" s="17"/>
-    </row>
-    <row r="8" spans="1:8" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="9"/>
+      <c r="F7" s="21"/>
+      <c r="G7" s="22"/>
+      <c r="H7" s="23"/>
+    </row>
+    <row r="8" spans="1:21" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="8"/>
       <c r="B8" s="7"/>
       <c r="C8" s="4"/>
       <c r="D8" s="4"/>
       <c r="E8" s="4"/>
-      <c r="F8" s="15"/>
-      <c r="G8" s="16"/>
-      <c r="H8" s="17"/>
-    </row>
-    <row r="9" spans="1:8" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="9"/>
+      <c r="F8" s="21"/>
+      <c r="G8" s="22"/>
+      <c r="H8" s="23"/>
+    </row>
+    <row r="9" spans="1:21" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="8"/>
       <c r="B9" s="7"/>
       <c r="C9" s="4"/>
       <c r="D9" s="4"/>
       <c r="E9" s="4"/>
-      <c r="F9" s="15"/>
-      <c r="G9" s="16"/>
-      <c r="H9" s="17"/>
-    </row>
-    <row r="10" spans="1:8" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="9"/>
+      <c r="F9" s="21"/>
+      <c r="G9" s="22"/>
+      <c r="H9" s="23"/>
+    </row>
+    <row r="10" spans="1:21" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="8"/>
       <c r="B10" s="7"/>
       <c r="C10" s="4"/>
       <c r="D10" s="4"/>
       <c r="E10" s="4"/>
-      <c r="F10" s="15"/>
-      <c r="G10" s="16"/>
-      <c r="H10" s="17"/>
-    </row>
-    <row r="11" spans="1:8" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="9"/>
+      <c r="F10" s="21"/>
+      <c r="G10" s="22"/>
+      <c r="H10" s="23"/>
+    </row>
+    <row r="11" spans="1:21" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="8"/>
       <c r="B11" s="7"/>
       <c r="C11" s="4"/>
       <c r="D11" s="4"/>
       <c r="E11" s="4"/>
-      <c r="F11" s="15"/>
-      <c r="G11" s="16"/>
-      <c r="H11" s="17"/>
-    </row>
-    <row r="12" spans="1:8" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="9"/>
+      <c r="F11" s="21"/>
+      <c r="G11" s="22"/>
+      <c r="H11" s="23"/>
+    </row>
+    <row r="12" spans="1:21" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="8"/>
       <c r="B12" s="7"/>
       <c r="C12" s="4"/>
       <c r="D12" s="4"/>
       <c r="E12" s="4"/>
-      <c r="F12" s="15"/>
-      <c r="G12" s="16"/>
-      <c r="H12" s="17"/>
-    </row>
-    <row r="13" spans="1:8" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="9"/>
+      <c r="F12" s="21"/>
+      <c r="G12" s="22"/>
+      <c r="H12" s="23"/>
+    </row>
+    <row r="13" spans="1:21" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="8"/>
       <c r="B13" s="7"/>
       <c r="C13" s="4"/>
       <c r="D13" s="4"/>
       <c r="E13" s="4"/>
-      <c r="F13" s="15"/>
-      <c r="G13" s="16"/>
-      <c r="H13" s="17"/>
-    </row>
-    <row r="14" spans="1:8" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="9"/>
+      <c r="F13" s="21"/>
+      <c r="G13" s="22"/>
+      <c r="H13" s="23"/>
+    </row>
+    <row r="14" spans="1:21" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="8"/>
       <c r="B14" s="7"/>
       <c r="C14" s="4"/>
       <c r="D14" s="4"/>
       <c r="E14" s="4"/>
-      <c r="F14" s="15"/>
-      <c r="G14" s="16"/>
-      <c r="H14" s="17"/>
-    </row>
-    <row r="15" spans="1:8" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="9"/>
+      <c r="F14" s="21"/>
+      <c r="G14" s="22"/>
+      <c r="H14" s="23"/>
+    </row>
+    <row r="15" spans="1:21" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="8"/>
       <c r="B15" s="7"/>
       <c r="C15" s="4"/>
       <c r="D15" s="4"/>
       <c r="E15" s="4"/>
-      <c r="F15" s="15"/>
-      <c r="G15" s="16"/>
-      <c r="H15" s="17"/>
-    </row>
-    <row r="16" spans="1:8" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="9"/>
+      <c r="F15" s="21"/>
+      <c r="G15" s="22"/>
+      <c r="H15" s="23"/>
+    </row>
+    <row r="16" spans="1:21" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="8"/>
       <c r="B16" s="7"/>
       <c r="C16" s="4"/>
       <c r="D16" s="4"/>
       <c r="E16" s="4"/>
-      <c r="F16" s="15"/>
-      <c r="G16" s="16"/>
-      <c r="H16" s="17"/>
-    </row>
-    <row r="17" spans="1:8" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="9"/>
+      <c r="F16" s="21"/>
+      <c r="G16" s="22"/>
+      <c r="H16" s="23"/>
+    </row>
+    <row r="17" spans="1:21" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="8"/>
       <c r="B17" s="7"/>
       <c r="C17" s="4"/>
       <c r="D17" s="4"/>
       <c r="E17" s="4"/>
-      <c r="F17" s="15"/>
-      <c r="G17" s="16"/>
-      <c r="H17" s="17"/>
-    </row>
-    <row r="18" spans="1:8" ht="48" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="10"/>
+      <c r="F17" s="21"/>
+      <c r="G17" s="22"/>
+      <c r="H17" s="23"/>
+    </row>
+    <row r="18" spans="1:21" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="8"/>
       <c r="B18" s="7"/>
       <c r="C18" s="4"/>
       <c r="D18" s="4"/>
       <c r="E18" s="4"/>
-      <c r="F18" s="15"/>
-      <c r="G18" s="16"/>
-      <c r="H18" s="17"/>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A19" s="8"/>
-      <c r="H19" s="2"/>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A20" s="1"/>
-      <c r="H20" s="2"/>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A21" s="1"/>
-      <c r="H21" s="2"/>
-    </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A22" s="1"/>
-      <c r="H22" s="2"/>
-    </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A23" s="1"/>
-      <c r="H23" s="2"/>
-    </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A24" s="1"/>
-      <c r="H24" s="2"/>
-    </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A25" s="1"/>
-      <c r="H25" s="2"/>
-    </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A26" s="1"/>
-      <c r="H26" s="2"/>
-    </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A27" s="1"/>
-      <c r="H27" s="2"/>
-    </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A28" s="1"/>
-      <c r="H28" s="2"/>
-    </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A29" s="1"/>
-      <c r="H29" s="2"/>
-    </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A30" s="1"/>
-      <c r="H30" s="2"/>
-    </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A31" s="1"/>
-      <c r="H31" s="11"/>
-    </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A32" s="1"/>
-      <c r="H32" s="2"/>
-    </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A33" s="1"/>
-      <c r="H33" s="2"/>
-    </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A34" s="1"/>
-      <c r="H34" s="2"/>
-    </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A35" s="1"/>
-      <c r="H35" s="2"/>
-    </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A36" s="1"/>
-      <c r="H36" s="2"/>
-    </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A37" s="1"/>
-      <c r="H37" s="2"/>
-    </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A38" s="1"/>
-      <c r="H38" s="2"/>
-    </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A39" s="1"/>
-      <c r="H39" s="2"/>
-    </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A40" s="1"/>
-      <c r="H40" s="2"/>
-    </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A41" s="1"/>
-      <c r="H41" s="2"/>
-    </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A42" s="1"/>
-      <c r="H42" s="2"/>
-    </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A43" s="1"/>
-      <c r="H43" s="2"/>
-    </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A44" s="1"/>
-      <c r="H44" s="2"/>
-    </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A45" s="1"/>
-      <c r="H45" s="2"/>
-    </row>
-    <row r="46" spans="1:8" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="12"/>
-      <c r="B46" s="13"/>
-      <c r="C46" s="13"/>
-      <c r="D46" s="13"/>
-      <c r="E46" s="13"/>
-      <c r="F46" s="13"/>
-      <c r="G46" s="13"/>
-      <c r="H46" s="14"/>
-    </row>
+      <c r="F18" s="21"/>
+      <c r="G18" s="22"/>
+      <c r="H18" s="23"/>
+    </row>
+    <row r="19" spans="1:21" ht="48" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="9"/>
+      <c r="B19" s="10"/>
+      <c r="C19" s="11"/>
+      <c r="D19" s="11"/>
+      <c r="E19" s="11"/>
+      <c r="F19" s="24"/>
+      <c r="G19" s="25"/>
+      <c r="H19" s="26"/>
+      <c r="K19" s="30"/>
+      <c r="L19" s="30"/>
+      <c r="M19" s="30"/>
+      <c r="N19" s="30"/>
+      <c r="O19" s="30"/>
+      <c r="P19" s="30"/>
+      <c r="Q19" s="30"/>
+      <c r="R19" s="30"/>
+      <c r="S19" s="30"/>
+      <c r="T19" s="30"/>
+      <c r="U19" s="30"/>
+    </row>
+    <row r="47" ht="16.5" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <mergeCells count="17">
-    <mergeCell ref="F14:H14"/>
+  <mergeCells count="20">
+    <mergeCell ref="K19:U19"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="F11:H11"/>
+    <mergeCell ref="F17:H17"/>
+    <mergeCell ref="T2:U2"/>
+    <mergeCell ref="J1:U1"/>
+    <mergeCell ref="F9:H9"/>
+    <mergeCell ref="F5:H5"/>
     <mergeCell ref="F18:H18"/>
     <mergeCell ref="F13:H13"/>
-    <mergeCell ref="B1:H1"/>
     <mergeCell ref="F8:H8"/>
+    <mergeCell ref="F10:H10"/>
     <mergeCell ref="F4:H4"/>
-    <mergeCell ref="F17:H17"/>
+    <mergeCell ref="F16:H16"/>
     <mergeCell ref="F12:H12"/>
     <mergeCell ref="F7:H7"/>
-    <mergeCell ref="F9:H9"/>
-    <mergeCell ref="F3:H3"/>
+    <mergeCell ref="F6:H6"/>
     <mergeCell ref="F15:H15"/>
-    <mergeCell ref="F11:H11"/>
-    <mergeCell ref="F16:H16"/>
-    <mergeCell ref="F10:H10"/>
-    <mergeCell ref="F6:H6"/>
-    <mergeCell ref="F5:H5"/>
+    <mergeCell ref="F19:H19"/>
+    <mergeCell ref="F14:H14"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.19685039370078741" right="0.19685039370078741" top="0.39370078740157483" bottom="0.39370078740157483" header="0.11811023622047249" footer="0.11811023622047249"/>
-  <pageSetup paperSize="9" scale="73" fitToHeight="2" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="68" fitToHeight="2" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Pequenas alterações no layout do grafico de chuva, pequenas alterações no relátorio em excel.
</commit_message>
<xml_diff>
--- a/templates/excel/ReportTemplate.xlsx
+++ b/templates/excel/ReportTemplate.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Emerson\Documents\MBA\Projetos\weather-forecast\templates\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A0CC8EF-2EA0-4675-B44A-9BE63B2778AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF0ECD78-8680-47C3-9475-EFAAD5085588}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,7 +17,7 @@
   </sheets>
   <definedNames>
     <definedName name="Abreviatura" hidden="1">#REF!</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Tempo Agora'!$A$1:$H$19,'Tempo Agora'!$J$1:$U$19</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Tempo Agora'!$A$1:$H$20,'Tempo Agora'!$J$1:$U$20</definedName>
     <definedName name="_xlnm.Recorder">#REF!</definedName>
     <definedName name="HSEAccidentsTable">OFFSET(#REF!,0,0,COUNTA(#REF!),5)</definedName>
     <definedName name="index_areaER">#REF!</definedName>
@@ -55,7 +55,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -112,6 +112,12 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <color theme="0" tint="-0.499984740745262"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -121,7 +127,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="16">
+  <borders count="17">
     <border>
       <left/>
       <right/>
@@ -308,6 +314,15 @@
         <color indexed="64"/>
       </top>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -317,7 +332,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
@@ -361,9 +376,6 @@
     <xf numFmtId="14" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -384,11 +396,24 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -747,26 +772,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:21" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="22"/>
-      <c r="B1" s="23"/>
-      <c r="C1" s="23"/>
-      <c r="D1" s="23"/>
-      <c r="E1" s="23"/>
-      <c r="F1" s="23"/>
-      <c r="G1" s="23"/>
-      <c r="H1" s="24"/>
-      <c r="J1" s="29"/>
-      <c r="K1" s="30"/>
-      <c r="L1" s="30"/>
-      <c r="M1" s="30"/>
-      <c r="N1" s="30"/>
-      <c r="O1" s="30"/>
-      <c r="P1" s="30"/>
-      <c r="Q1" s="30"/>
-      <c r="R1" s="30"/>
-      <c r="S1" s="30"/>
-      <c r="T1" s="30"/>
-      <c r="U1" s="30"/>
+      <c r="A1" s="21"/>
+      <c r="B1" s="22"/>
+      <c r="C1" s="22"/>
+      <c r="D1" s="22"/>
+      <c r="E1" s="22"/>
+      <c r="F1" s="22"/>
+      <c r="G1" s="22"/>
+      <c r="H1" s="23"/>
+      <c r="J1" s="28"/>
+      <c r="K1" s="29"/>
+      <c r="L1" s="29"/>
+      <c r="M1" s="29"/>
+      <c r="N1" s="29"/>
+      <c r="O1" s="29"/>
+      <c r="P1" s="29"/>
+      <c r="Q1" s="29"/>
+      <c r="R1" s="29"/>
+      <c r="S1" s="29"/>
+      <c r="T1" s="29"/>
+      <c r="U1" s="29"/>
     </row>
     <row r="2" spans="1:21" ht="51" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1"/>
@@ -781,11 +806,16 @@
       <c r="L2" s="17"/>
       <c r="M2" s="18"/>
       <c r="S2" s="12"/>
-      <c r="T2" s="28"/>
-      <c r="U2" s="28"/>
+      <c r="T2" s="27"/>
+      <c r="U2" s="27"/>
     </row>
     <row r="3" spans="1:21" ht="242.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
+      <c r="C3" s="31"/>
+      <c r="D3" s="31"/>
+      <c r="E3" s="31"/>
+      <c r="F3" s="31"/>
+      <c r="G3" s="31"/>
       <c r="H3" s="2"/>
     </row>
     <row r="4" spans="1:21" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -802,11 +832,11 @@
       <c r="E4" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="F4" s="31" t="s">
+      <c r="F4" s="30" t="s">
         <v>4</v>
       </c>
-      <c r="G4" s="26"/>
-      <c r="H4" s="27"/>
+      <c r="G4" s="25"/>
+      <c r="H4" s="26"/>
     </row>
     <row r="5" spans="1:21" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="8"/>
@@ -814,9 +844,9 @@
       <c r="C5" s="4"/>
       <c r="D5" s="4"/>
       <c r="E5" s="4"/>
-      <c r="F5" s="25"/>
-      <c r="G5" s="26"/>
-      <c r="H5" s="27"/>
+      <c r="F5" s="24"/>
+      <c r="G5" s="25"/>
+      <c r="H5" s="26"/>
     </row>
     <row r="6" spans="1:21" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="8"/>
@@ -824,9 +854,9 @@
       <c r="C6" s="4"/>
       <c r="D6" s="4"/>
       <c r="E6" s="4"/>
-      <c r="F6" s="25"/>
-      <c r="G6" s="26"/>
-      <c r="H6" s="27"/>
+      <c r="F6" s="24"/>
+      <c r="G6" s="25"/>
+      <c r="H6" s="26"/>
     </row>
     <row r="7" spans="1:21" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="8"/>
@@ -834,9 +864,9 @@
       <c r="C7" s="4"/>
       <c r="D7" s="4"/>
       <c r="E7" s="4"/>
-      <c r="F7" s="25"/>
-      <c r="G7" s="26"/>
-      <c r="H7" s="27"/>
+      <c r="F7" s="24"/>
+      <c r="G7" s="25"/>
+      <c r="H7" s="26"/>
     </row>
     <row r="8" spans="1:21" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="8"/>
@@ -844,9 +874,9 @@
       <c r="C8" s="4"/>
       <c r="D8" s="4"/>
       <c r="E8" s="4"/>
-      <c r="F8" s="25"/>
-      <c r="G8" s="26"/>
-      <c r="H8" s="27"/>
+      <c r="F8" s="24"/>
+      <c r="G8" s="25"/>
+      <c r="H8" s="26"/>
     </row>
     <row r="9" spans="1:21" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="8"/>
@@ -854,9 +884,9 @@
       <c r="C9" s="4"/>
       <c r="D9" s="4"/>
       <c r="E9" s="4"/>
-      <c r="F9" s="25"/>
-      <c r="G9" s="26"/>
-      <c r="H9" s="27"/>
+      <c r="F9" s="24"/>
+      <c r="G9" s="25"/>
+      <c r="H9" s="26"/>
     </row>
     <row r="10" spans="1:21" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="8"/>
@@ -864,9 +894,9 @@
       <c r="C10" s="4"/>
       <c r="D10" s="4"/>
       <c r="E10" s="4"/>
-      <c r="F10" s="25"/>
-      <c r="G10" s="26"/>
-      <c r="H10" s="27"/>
+      <c r="F10" s="24"/>
+      <c r="G10" s="25"/>
+      <c r="H10" s="26"/>
     </row>
     <row r="11" spans="1:21" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="8"/>
@@ -874,9 +904,9 @@
       <c r="C11" s="4"/>
       <c r="D11" s="4"/>
       <c r="E11" s="4"/>
-      <c r="F11" s="25"/>
-      <c r="G11" s="26"/>
-      <c r="H11" s="27"/>
+      <c r="F11" s="24"/>
+      <c r="G11" s="25"/>
+      <c r="H11" s="26"/>
     </row>
     <row r="12" spans="1:21" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="8"/>
@@ -884,9 +914,9 @@
       <c r="C12" s="4"/>
       <c r="D12" s="4"/>
       <c r="E12" s="4"/>
-      <c r="F12" s="25"/>
-      <c r="G12" s="26"/>
-      <c r="H12" s="27"/>
+      <c r="F12" s="24"/>
+      <c r="G12" s="25"/>
+      <c r="H12" s="26"/>
     </row>
     <row r="13" spans="1:21" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="8"/>
@@ -894,9 +924,9 @@
       <c r="C13" s="4"/>
       <c r="D13" s="4"/>
       <c r="E13" s="4"/>
-      <c r="F13" s="25"/>
-      <c r="G13" s="26"/>
-      <c r="H13" s="27"/>
+      <c r="F13" s="24"/>
+      <c r="G13" s="25"/>
+      <c r="H13" s="26"/>
     </row>
     <row r="14" spans="1:21" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="8"/>
@@ -904,9 +934,9 @@
       <c r="C14" s="4"/>
       <c r="D14" s="4"/>
       <c r="E14" s="4"/>
-      <c r="F14" s="25"/>
-      <c r="G14" s="26"/>
-      <c r="H14" s="27"/>
+      <c r="F14" s="24"/>
+      <c r="G14" s="25"/>
+      <c r="H14" s="26"/>
     </row>
     <row r="15" spans="1:21" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="8"/>
@@ -914,9 +944,9 @@
       <c r="C15" s="4"/>
       <c r="D15" s="4"/>
       <c r="E15" s="4"/>
-      <c r="F15" s="25"/>
-      <c r="G15" s="26"/>
-      <c r="H15" s="27"/>
+      <c r="F15" s="24"/>
+      <c r="G15" s="25"/>
+      <c r="H15" s="26"/>
     </row>
     <row r="16" spans="1:21" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="8"/>
@@ -924,9 +954,9 @@
       <c r="C16" s="4"/>
       <c r="D16" s="4"/>
       <c r="E16" s="4"/>
-      <c r="F16" s="25"/>
-      <c r="G16" s="26"/>
-      <c r="H16" s="27"/>
+      <c r="F16" s="24"/>
+      <c r="G16" s="25"/>
+      <c r="H16" s="26"/>
     </row>
     <row r="17" spans="1:21" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="8"/>
@@ -934,9 +964,9 @@
       <c r="C17" s="4"/>
       <c r="D17" s="4"/>
       <c r="E17" s="4"/>
-      <c r="F17" s="25"/>
-      <c r="G17" s="26"/>
-      <c r="H17" s="27"/>
+      <c r="F17" s="24"/>
+      <c r="G17" s="25"/>
+      <c r="H17" s="26"/>
     </row>
     <row r="18" spans="1:21" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="8"/>
@@ -944,9 +974,9 @@
       <c r="C18" s="4"/>
       <c r="D18" s="4"/>
       <c r="E18" s="4"/>
-      <c r="F18" s="25"/>
-      <c r="G18" s="26"/>
-      <c r="H18" s="27"/>
+      <c r="F18" s="24"/>
+      <c r="G18" s="25"/>
+      <c r="H18" s="26"/>
     </row>
     <row r="19" spans="1:21" ht="48" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="9"/>
@@ -957,26 +987,39 @@
       <c r="F19" s="32"/>
       <c r="G19" s="33"/>
       <c r="H19" s="34"/>
-      <c r="K19" s="21"/>
-      <c r="L19" s="21"/>
-      <c r="M19" s="21"/>
-      <c r="N19" s="21"/>
-      <c r="O19" s="21"/>
-      <c r="P19" s="21"/>
-      <c r="Q19" s="21"/>
-      <c r="R19" s="21"/>
-      <c r="S19" s="21"/>
-      <c r="T19" s="21"/>
-      <c r="U19" s="21"/>
+      <c r="K19" s="35"/>
+      <c r="L19" s="35"/>
+      <c r="M19" s="35"/>
+      <c r="N19" s="35"/>
+      <c r="O19" s="35"/>
+      <c r="P19" s="35"/>
+      <c r="Q19" s="35"/>
+      <c r="R19" s="35"/>
+      <c r="S19" s="35"/>
+      <c r="T19" s="35"/>
+      <c r="U19" s="35"/>
+    </row>
+    <row r="20" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="F20" s="36"/>
+      <c r="G20" s="36"/>
+      <c r="H20" s="36"/>
+      <c r="S20" s="37"/>
+      <c r="T20" s="37"/>
+      <c r="U20" s="37"/>
+    </row>
+    <row r="24" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="H24" s="38"/>
     </row>
     <row r="47" ht="16.5" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <mergeCells count="20">
-    <mergeCell ref="F6:H6"/>
+  <mergeCells count="23">
+    <mergeCell ref="F20:H20"/>
+    <mergeCell ref="S20:U20"/>
     <mergeCell ref="F15:H15"/>
     <mergeCell ref="F19:H19"/>
     <mergeCell ref="F14:H14"/>
     <mergeCell ref="K19:U19"/>
+    <mergeCell ref="F18:H18"/>
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="F11:H11"/>
     <mergeCell ref="F17:H17"/>
@@ -984,7 +1027,6 @@
     <mergeCell ref="J1:U1"/>
     <mergeCell ref="F9:H9"/>
     <mergeCell ref="F5:H5"/>
-    <mergeCell ref="F18:H18"/>
     <mergeCell ref="F13:H13"/>
     <mergeCell ref="F8:H8"/>
     <mergeCell ref="F10:H10"/>
@@ -992,6 +1034,8 @@
     <mergeCell ref="F16:H16"/>
     <mergeCell ref="F12:H12"/>
     <mergeCell ref="F7:H7"/>
+    <mergeCell ref="C3:G3"/>
+    <mergeCell ref="F6:H6"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.19685039370078741" right="0.19685039370078741" top="0.39370078740157483" bottom="0.39370078740157483" header="0.11811023622047249" footer="0.11811023622047249"/>

</xml_diff>

<commit_message>
Alteração da Págiona Sobre, pequena alteracao no layout do relatorio, e cache nos dados do infoclima
</commit_message>
<xml_diff>
--- a/templates/excel/ReportTemplate.xlsx
+++ b/templates/excel/ReportTemplate.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Emerson\Documents\MBA\Projetos\weather-forecast\templates\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBE5644E-6EC0-49CD-98D7-43C1E4377294}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{449A72F4-7905-4A3A-A3CE-E6D329667AC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="23280" windowHeight="12480" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tempo Agora" sheetId="1" r:id="rId1"/>
@@ -608,7 +608,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
@@ -650,22 +650,15 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -678,7 +671,13 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1036,7 +1035,7 @@
     <col min="21" max="21" width="6.625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" s="33" customFormat="1" ht="48.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:21" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="5"/>
       <c r="C1" s="5"/>
       <c r="D1" s="5"/>
@@ -1060,11 +1059,11 @@
       <c r="L2" s="2"/>
       <c r="M2" s="3"/>
       <c r="S2" s="1"/>
-      <c r="T2" s="19"/>
+      <c r="T2" s="30"/>
       <c r="U2" s="20"/>
     </row>
     <row r="3" spans="1:21" ht="242.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C3" s="26"/>
+      <c r="C3" s="19"/>
       <c r="D3" s="20"/>
       <c r="E3" s="20"/>
       <c r="F3" s="20"/>
@@ -1084,11 +1083,11 @@
       <c r="E4" s="18" t="s">
         <v>110</v>
       </c>
-      <c r="F4" s="21" t="s">
+      <c r="F4" s="31" t="s">
         <v>111</v>
       </c>
       <c r="G4" s="22"/>
-      <c r="H4" s="23"/>
+      <c r="H4" s="32"/>
     </row>
     <row r="5" spans="1:21" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="11"/>
@@ -1096,9 +1095,9 @@
       <c r="C5" s="13"/>
       <c r="D5" s="13"/>
       <c r="E5" s="13"/>
-      <c r="F5" s="24"/>
+      <c r="F5" s="21"/>
       <c r="G5" s="22"/>
-      <c r="H5" s="25"/>
+      <c r="H5" s="23"/>
     </row>
     <row r="6" spans="1:21" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="11"/>
@@ -1106,9 +1105,9 @@
       <c r="C6" s="13"/>
       <c r="D6" s="13"/>
       <c r="E6" s="13"/>
-      <c r="F6" s="24"/>
+      <c r="F6" s="21"/>
       <c r="G6" s="22"/>
-      <c r="H6" s="25"/>
+      <c r="H6" s="23"/>
     </row>
     <row r="7" spans="1:21" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="11"/>
@@ -1116,9 +1115,9 @@
       <c r="C7" s="13"/>
       <c r="D7" s="13"/>
       <c r="E7" s="13"/>
-      <c r="F7" s="24"/>
+      <c r="F7" s="21"/>
       <c r="G7" s="22"/>
-      <c r="H7" s="25"/>
+      <c r="H7" s="23"/>
     </row>
     <row r="8" spans="1:21" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="11"/>
@@ -1126,9 +1125,9 @@
       <c r="C8" s="13"/>
       <c r="D8" s="13"/>
       <c r="E8" s="13"/>
-      <c r="F8" s="24"/>
+      <c r="F8" s="21"/>
       <c r="G8" s="22"/>
-      <c r="H8" s="25"/>
+      <c r="H8" s="23"/>
     </row>
     <row r="9" spans="1:21" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="11"/>
@@ -1136,9 +1135,9 @@
       <c r="C9" s="13"/>
       <c r="D9" s="13"/>
       <c r="E9" s="13"/>
-      <c r="F9" s="24"/>
+      <c r="F9" s="21"/>
       <c r="G9" s="22"/>
-      <c r="H9" s="25"/>
+      <c r="H9" s="23"/>
     </row>
     <row r="10" spans="1:21" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="11"/>
@@ -1146,9 +1145,9 @@
       <c r="C10" s="13"/>
       <c r="D10" s="13"/>
       <c r="E10" s="13"/>
-      <c r="F10" s="24"/>
+      <c r="F10" s="21"/>
       <c r="G10" s="22"/>
-      <c r="H10" s="25"/>
+      <c r="H10" s="23"/>
     </row>
     <row r="11" spans="1:21" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="11"/>
@@ -1156,9 +1155,9 @@
       <c r="C11" s="13"/>
       <c r="D11" s="13"/>
       <c r="E11" s="13"/>
-      <c r="F11" s="24"/>
+      <c r="F11" s="21"/>
       <c r="G11" s="22"/>
-      <c r="H11" s="25"/>
+      <c r="H11" s="23"/>
     </row>
     <row r="12" spans="1:21" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="11"/>
@@ -1166,9 +1165,9 @@
       <c r="C12" s="13"/>
       <c r="D12" s="13"/>
       <c r="E12" s="13"/>
-      <c r="F12" s="24"/>
+      <c r="F12" s="21"/>
       <c r="G12" s="22"/>
-      <c r="H12" s="25"/>
+      <c r="H12" s="23"/>
     </row>
     <row r="13" spans="1:21" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="11"/>
@@ -1176,9 +1175,9 @@
       <c r="C13" s="13"/>
       <c r="D13" s="13"/>
       <c r="E13" s="13"/>
-      <c r="F13" s="24"/>
+      <c r="F13" s="21"/>
       <c r="G13" s="22"/>
-      <c r="H13" s="25"/>
+      <c r="H13" s="23"/>
     </row>
     <row r="14" spans="1:21" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="11"/>
@@ -1186,9 +1185,9 @@
       <c r="C14" s="13"/>
       <c r="D14" s="13"/>
       <c r="E14" s="13"/>
-      <c r="F14" s="24"/>
+      <c r="F14" s="21"/>
       <c r="G14" s="22"/>
-      <c r="H14" s="25"/>
+      <c r="H14" s="23"/>
     </row>
     <row r="15" spans="1:21" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="11"/>
@@ -1196,9 +1195,9 @@
       <c r="C15" s="13"/>
       <c r="D15" s="13"/>
       <c r="E15" s="13"/>
-      <c r="F15" s="24"/>
+      <c r="F15" s="21"/>
       <c r="G15" s="22"/>
-      <c r="H15" s="25"/>
+      <c r="H15" s="23"/>
     </row>
     <row r="16" spans="1:21" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="11"/>
@@ -1206,9 +1205,9 @@
       <c r="C16" s="13"/>
       <c r="D16" s="13"/>
       <c r="E16" s="13"/>
-      <c r="F16" s="24"/>
+      <c r="F16" s="21"/>
       <c r="G16" s="22"/>
-      <c r="H16" s="25"/>
+      <c r="H16" s="23"/>
     </row>
     <row r="17" spans="1:21" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="11"/>
@@ -1216,9 +1215,9 @@
       <c r="C17" s="13"/>
       <c r="D17" s="13"/>
       <c r="E17" s="13"/>
-      <c r="F17" s="24"/>
+      <c r="F17" s="21"/>
       <c r="G17" s="22"/>
-      <c r="H17" s="25"/>
+      <c r="H17" s="23"/>
     </row>
     <row r="18" spans="1:21" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="11"/>
@@ -1226,9 +1225,9 @@
       <c r="C18" s="13"/>
       <c r="D18" s="13"/>
       <c r="E18" s="13"/>
-      <c r="F18" s="24"/>
+      <c r="F18" s="21"/>
       <c r="G18" s="22"/>
-      <c r="H18" s="25"/>
+      <c r="H18" s="23"/>
     </row>
     <row r="19" spans="1:21" ht="48" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="14"/>
@@ -1236,10 +1235,10 @@
       <c r="C19" s="16"/>
       <c r="D19" s="16"/>
       <c r="E19" s="16"/>
-      <c r="F19" s="27"/>
-      <c r="G19" s="28"/>
-      <c r="H19" s="29"/>
-      <c r="K19" s="32"/>
+      <c r="F19" s="24"/>
+      <c r="G19" s="25"/>
+      <c r="H19" s="26"/>
+      <c r="K19" s="29"/>
       <c r="L19" s="20"/>
       <c r="M19" s="20"/>
       <c r="N19" s="20"/>
@@ -1252,24 +1251,16 @@
       <c r="U19" s="20"/>
     </row>
     <row r="20" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="F20" s="30"/>
-      <c r="G20" s="31"/>
-      <c r="H20" s="31"/>
-      <c r="S20" s="26"/>
+      <c r="F20" s="27"/>
+      <c r="G20" s="28"/>
+      <c r="H20" s="28"/>
+      <c r="S20" s="19"/>
       <c r="T20" s="20"/>
       <c r="U20" s="20"/>
     </row>
     <row r="47" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="21">
-    <mergeCell ref="S20:U20"/>
-    <mergeCell ref="F14:H14"/>
-    <mergeCell ref="F19:H19"/>
-    <mergeCell ref="F15:H15"/>
-    <mergeCell ref="F20:H20"/>
-    <mergeCell ref="F18:H18"/>
-    <mergeCell ref="K19:U19"/>
-    <mergeCell ref="F17:H17"/>
     <mergeCell ref="T2:U2"/>
     <mergeCell ref="F4:H4"/>
     <mergeCell ref="F11:H11"/>
@@ -1283,6 +1274,14 @@
     <mergeCell ref="F9:H9"/>
     <mergeCell ref="F5:H5"/>
     <mergeCell ref="F8:H8"/>
+    <mergeCell ref="S20:U20"/>
+    <mergeCell ref="F14:H14"/>
+    <mergeCell ref="F19:H19"/>
+    <mergeCell ref="F15:H15"/>
+    <mergeCell ref="F20:H20"/>
+    <mergeCell ref="F18:H18"/>
+    <mergeCell ref="K19:U19"/>
+    <mergeCell ref="F17:H17"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.19685039370078741" right="0.19685039370078741" top="0.39370078740157483" bottom="0.39370078740157483" header="0.11811023622047245" footer="0.11811023622047245"/>

</xml_diff>

<commit_message>
Correção da inmet_api, alterações para o tratamento das imagens do INMET
</commit_message>
<xml_diff>
--- a/templates/excel/ReportTemplate.xlsx
+++ b/templates/excel/ReportTemplate.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr codeName="EstaPastaDeTrabalho" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Emerson\Documents\MBA\Projetos\weather-forecast\templates\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9AA9A4B-6014-4D67-804E-FBD948A9A216}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6F1F72A-6F0A-4AFB-8F71-F86E7F40ED2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="23280" windowHeight="12480" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tempo Agora" sheetId="1" r:id="rId1"/>
@@ -286,7 +286,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
@@ -328,22 +328,18 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -356,6 +352,13 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -737,15 +740,16 @@
       <c r="L2" s="2"/>
       <c r="M2" s="3"/>
       <c r="S2" s="1"/>
-      <c r="T2" s="19"/>
-      <c r="U2" s="20"/>
+      <c r="T2" s="31"/>
+      <c r="U2" s="21"/>
     </row>
     <row r="3" spans="1:21" ht="242.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C3" s="26"/>
-      <c r="D3" s="20"/>
-      <c r="E3" s="20"/>
-      <c r="F3" s="20"/>
-      <c r="G3" s="20"/>
+      <c r="C3" s="20"/>
+      <c r="D3" s="21"/>
+      <c r="E3" s="21"/>
+      <c r="F3" s="21"/>
+      <c r="G3" s="21"/>
+      <c r="H3" s="19"/>
     </row>
     <row r="4" spans="1:21" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="10"/>
@@ -761,11 +765,11 @@
       <c r="E4" s="18" t="s">
         <v>3</v>
       </c>
-      <c r="F4" s="21" t="s">
+      <c r="F4" s="32" t="s">
         <v>4</v>
       </c>
-      <c r="G4" s="22"/>
-      <c r="H4" s="23"/>
+      <c r="G4" s="23"/>
+      <c r="H4" s="33"/>
     </row>
     <row r="5" spans="1:21" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="11"/>
@@ -773,9 +777,9 @@
       <c r="C5" s="13"/>
       <c r="D5" s="13"/>
       <c r="E5" s="13"/>
-      <c r="F5" s="24"/>
-      <c r="G5" s="22"/>
-      <c r="H5" s="25"/>
+      <c r="F5" s="22"/>
+      <c r="G5" s="23"/>
+      <c r="H5" s="24"/>
     </row>
     <row r="6" spans="1:21" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="11"/>
@@ -783,9 +787,9 @@
       <c r="C6" s="13"/>
       <c r="D6" s="13"/>
       <c r="E6" s="13"/>
-      <c r="F6" s="24"/>
-      <c r="G6" s="22"/>
-      <c r="H6" s="25"/>
+      <c r="F6" s="22"/>
+      <c r="G6" s="23"/>
+      <c r="H6" s="24"/>
     </row>
     <row r="7" spans="1:21" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="11"/>
@@ -793,9 +797,9 @@
       <c r="C7" s="13"/>
       <c r="D7" s="13"/>
       <c r="E7" s="13"/>
-      <c r="F7" s="24"/>
-      <c r="G7" s="22"/>
-      <c r="H7" s="25"/>
+      <c r="F7" s="22"/>
+      <c r="G7" s="23"/>
+      <c r="H7" s="24"/>
     </row>
     <row r="8" spans="1:21" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="11"/>
@@ -803,9 +807,9 @@
       <c r="C8" s="13"/>
       <c r="D8" s="13"/>
       <c r="E8" s="13"/>
-      <c r="F8" s="24"/>
-      <c r="G8" s="22"/>
-      <c r="H8" s="25"/>
+      <c r="F8" s="22"/>
+      <c r="G8" s="23"/>
+      <c r="H8" s="24"/>
     </row>
     <row r="9" spans="1:21" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="11"/>
@@ -813,9 +817,9 @@
       <c r="C9" s="13"/>
       <c r="D9" s="13"/>
       <c r="E9" s="13"/>
-      <c r="F9" s="24"/>
-      <c r="G9" s="22"/>
-      <c r="H9" s="25"/>
+      <c r="F9" s="22"/>
+      <c r="G9" s="23"/>
+      <c r="H9" s="24"/>
     </row>
     <row r="10" spans="1:21" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="11"/>
@@ -823,9 +827,9 @@
       <c r="C10" s="13"/>
       <c r="D10" s="13"/>
       <c r="E10" s="13"/>
-      <c r="F10" s="24"/>
-      <c r="G10" s="22"/>
-      <c r="H10" s="25"/>
+      <c r="F10" s="22"/>
+      <c r="G10" s="23"/>
+      <c r="H10" s="24"/>
     </row>
     <row r="11" spans="1:21" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="11"/>
@@ -833,9 +837,9 @@
       <c r="C11" s="13"/>
       <c r="D11" s="13"/>
       <c r="E11" s="13"/>
-      <c r="F11" s="24"/>
-      <c r="G11" s="22"/>
-      <c r="H11" s="25"/>
+      <c r="F11" s="22"/>
+      <c r="G11" s="23"/>
+      <c r="H11" s="24"/>
     </row>
     <row r="12" spans="1:21" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="11"/>
@@ -843,9 +847,9 @@
       <c r="C12" s="13"/>
       <c r="D12" s="13"/>
       <c r="E12" s="13"/>
-      <c r="F12" s="24"/>
-      <c r="G12" s="22"/>
-      <c r="H12" s="25"/>
+      <c r="F12" s="22"/>
+      <c r="G12" s="23"/>
+      <c r="H12" s="24"/>
     </row>
     <row r="13" spans="1:21" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="11"/>
@@ -853,9 +857,9 @@
       <c r="C13" s="13"/>
       <c r="D13" s="13"/>
       <c r="E13" s="13"/>
-      <c r="F13" s="24"/>
-      <c r="G13" s="22"/>
-      <c r="H13" s="25"/>
+      <c r="F13" s="22"/>
+      <c r="G13" s="23"/>
+      <c r="H13" s="24"/>
     </row>
     <row r="14" spans="1:21" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="11"/>
@@ -863,9 +867,9 @@
       <c r="C14" s="13"/>
       <c r="D14" s="13"/>
       <c r="E14" s="13"/>
-      <c r="F14" s="24"/>
-      <c r="G14" s="22"/>
-      <c r="H14" s="25"/>
+      <c r="F14" s="22"/>
+      <c r="G14" s="23"/>
+      <c r="H14" s="24"/>
     </row>
     <row r="15" spans="1:21" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="11"/>
@@ -873,9 +877,9 @@
       <c r="C15" s="13"/>
       <c r="D15" s="13"/>
       <c r="E15" s="13"/>
-      <c r="F15" s="24"/>
-      <c r="G15" s="22"/>
-      <c r="H15" s="25"/>
+      <c r="F15" s="22"/>
+      <c r="G15" s="23"/>
+      <c r="H15" s="24"/>
     </row>
     <row r="16" spans="1:21" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="11"/>
@@ -883,9 +887,9 @@
       <c r="C16" s="13"/>
       <c r="D16" s="13"/>
       <c r="E16" s="13"/>
-      <c r="F16" s="24"/>
-      <c r="G16" s="22"/>
-      <c r="H16" s="25"/>
+      <c r="F16" s="22"/>
+      <c r="G16" s="23"/>
+      <c r="H16" s="24"/>
     </row>
     <row r="17" spans="1:21" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="11"/>
@@ -893,9 +897,9 @@
       <c r="C17" s="13"/>
       <c r="D17" s="13"/>
       <c r="E17" s="13"/>
-      <c r="F17" s="24"/>
-      <c r="G17" s="22"/>
-      <c r="H17" s="25"/>
+      <c r="F17" s="22"/>
+      <c r="G17" s="23"/>
+      <c r="H17" s="24"/>
     </row>
     <row r="18" spans="1:21" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="11"/>
@@ -903,9 +907,9 @@
       <c r="C18" s="13"/>
       <c r="D18" s="13"/>
       <c r="E18" s="13"/>
-      <c r="F18" s="24"/>
-      <c r="G18" s="22"/>
-      <c r="H18" s="25"/>
+      <c r="F18" s="22"/>
+      <c r="G18" s="23"/>
+      <c r="H18" s="24"/>
     </row>
     <row r="19" spans="1:21" ht="48" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="14"/>
@@ -913,40 +917,32 @@
       <c r="C19" s="16"/>
       <c r="D19" s="16"/>
       <c r="E19" s="16"/>
-      <c r="F19" s="27"/>
-      <c r="G19" s="28"/>
-      <c r="H19" s="29"/>
-      <c r="K19" s="32"/>
-      <c r="L19" s="20"/>
-      <c r="M19" s="20"/>
-      <c r="N19" s="20"/>
-      <c r="O19" s="20"/>
-      <c r="P19" s="20"/>
-      <c r="Q19" s="20"/>
-      <c r="R19" s="20"/>
-      <c r="S19" s="20"/>
-      <c r="T19" s="20"/>
-      <c r="U19" s="20"/>
+      <c r="F19" s="25"/>
+      <c r="G19" s="26"/>
+      <c r="H19" s="27"/>
+      <c r="K19" s="30"/>
+      <c r="L19" s="21"/>
+      <c r="M19" s="21"/>
+      <c r="N19" s="21"/>
+      <c r="O19" s="21"/>
+      <c r="P19" s="21"/>
+      <c r="Q19" s="21"/>
+      <c r="R19" s="21"/>
+      <c r="S19" s="21"/>
+      <c r="T19" s="21"/>
+      <c r="U19" s="21"/>
     </row>
     <row r="20" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="F20" s="30"/>
-      <c r="G20" s="31"/>
-      <c r="H20" s="31"/>
-      <c r="S20" s="26"/>
-      <c r="T20" s="20"/>
-      <c r="U20" s="20"/>
+      <c r="F20" s="28"/>
+      <c r="G20" s="29"/>
+      <c r="H20" s="29"/>
+      <c r="S20" s="20"/>
+      <c r="T20" s="21"/>
+      <c r="U20" s="21"/>
     </row>
     <row r="47" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="21">
-    <mergeCell ref="S20:U20"/>
-    <mergeCell ref="F14:H14"/>
-    <mergeCell ref="F19:H19"/>
-    <mergeCell ref="F15:H15"/>
-    <mergeCell ref="F20:H20"/>
-    <mergeCell ref="F18:H18"/>
-    <mergeCell ref="K19:U19"/>
-    <mergeCell ref="F17:H17"/>
     <mergeCell ref="T2:U2"/>
     <mergeCell ref="F4:H4"/>
     <mergeCell ref="F11:H11"/>
@@ -960,6 +956,14 @@
     <mergeCell ref="F9:H9"/>
     <mergeCell ref="F5:H5"/>
     <mergeCell ref="F8:H8"/>
+    <mergeCell ref="S20:U20"/>
+    <mergeCell ref="F14:H14"/>
+    <mergeCell ref="F19:H19"/>
+    <mergeCell ref="F15:H15"/>
+    <mergeCell ref="F20:H20"/>
+    <mergeCell ref="F18:H18"/>
+    <mergeCell ref="K19:U19"/>
+    <mergeCell ref="F17:H17"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.19685039370078741" right="0.19685039370078741" top="0.39370078740157483" bottom="0.39370078740157483" header="0.11811023622047245" footer="0.11811023622047245"/>

</xml_diff>